<commit_message>
chore: sync local changes
</commit_message>
<xml_diff>
--- a/组织通灵计算器.xlsx
+++ b/组织通灵计算器.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\utility\naruto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADEC25F-11A9-4BD9-92E5-1185EC0CFB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E547ACF2-0338-4C42-B47D-4E4EC12CF17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4485" yWindow="210" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="计算器" sheetId="1" r:id="rId1"/>
@@ -291,60 +291,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -620,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="0.42578125" customWidth="1"/>
@@ -632,215 +629,207 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="3" customHeight="1">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" spans="1:6" ht="21">
-      <c r="A2" s="3"/>
-      <c r="B2" s="12" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="14"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="15" t="s">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="E3" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="16"/>
+      <c r="F3" s="13"/>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="10"/>
+      <c r="A4" s="2"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="8"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="2"/>
+      <c r="B5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="5">
         <v>1</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="5">
         <v>0</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="8" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="10"/>
+      <c r="A6" s="2"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="6"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="8"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="2"/>
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="5">
         <v>181</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="11"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="8"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="10"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="6"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="2"/>
+      <c r="B9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="9">
+      <c r="C9" s="7">
         <f>数据源!F3-数据源!F2</f>
         <v>312000</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="10"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="8"/>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="10"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="6"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="3"/>
-      <c r="B11" s="17" t="s">
+      <c r="A11" s="2"/>
+      <c r="B11" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="2"/>
+      <c r="B12" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="7">
-        <v>6891</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="C12" s="5">
+        <v>7311</v>
+      </c>
+      <c r="D12" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="10"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="2"/>
+      <c r="B13" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="5">
         <v>1080</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="10"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="2"/>
+      <c r="B14" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="7">
-        <v>82</v>
-      </c>
-      <c r="D14" s="6" t="s">
+      <c r="C14" s="5">
+        <v>53</v>
+      </c>
+      <c r="D14" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="10"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="10"/>
+      <c r="A15" s="2"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="6"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="2"/>
+      <c r="B16" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="9">
+      <c r="C16" s="7">
         <f>C9-数据源!F4</f>
-        <v>-15820</v>
-      </c>
-      <c r="D16" s="6" t="s">
+        <v>4780</v>
+      </c>
+      <c r="D16" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="10"/>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="10"/>
-    </row>
-    <row r="18" spans="1:8" ht="14.25" customHeight="1">
-      <c r="A18" s="3"/>
-      <c r="B18" s="20" t="s">
+      <c r="E16" s="4"/>
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="2"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" spans="1:6" ht="14.25" customHeight="1">
+      <c r="A18" s="2"/>
+      <c r="B18" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="22"/>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="3"/>
-      <c r="B19" s="23" t="s">
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="19"/>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="2"/>
+      <c r="B19" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="25"/>
-      <c r="H19" s="6"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="22"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="LxYxc3SqIMCjJ61HfANHyTErF0T2fz/xFXqD4O6o5OpCyOCf0MT3x1XQyTazSScVOupE53X0tK9zfjHlAiSlUw==" saltValue="TxTS0gAGdGdwE9quylhnVw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
@@ -929,7 +918,7 @@
       </c>
       <c r="F4">
         <f>计算器!C12*20+计算器!C13*100+计算器!C14*1000</f>
-        <v>327820</v>
+        <v>307220</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -3312,7 +3301,7 @@
       <c r="A203" s="1">
         <v>202</v>
       </c>
-      <c r="B203" s="2">
+      <c r="B203" s="1">
         <v>4000</v>
       </c>
       <c r="C203" s="1">
@@ -3324,7 +3313,7 @@
       <c r="A204" s="1">
         <v>203</v>
       </c>
-      <c r="B204" s="2">
+      <c r="B204" s="1">
         <v>4000</v>
       </c>
       <c r="C204" s="1">
@@ -3336,7 +3325,7 @@
       <c r="A205" s="1">
         <v>204</v>
       </c>
-      <c r="B205" s="2">
+      <c r="B205" s="1">
         <v>4000</v>
       </c>
       <c r="C205" s="1">
@@ -3348,7 +3337,7 @@
       <c r="A206" s="1">
         <v>205</v>
       </c>
-      <c r="B206" s="2">
+      <c r="B206" s="1">
         <v>4000</v>
       </c>
       <c r="C206" s="1">
@@ -3360,7 +3349,7 @@
       <c r="A207" s="1">
         <v>206</v>
       </c>
-      <c r="B207" s="2">
+      <c r="B207" s="1">
         <v>4000</v>
       </c>
       <c r="C207" s="1">
@@ -3372,7 +3361,7 @@
       <c r="A208" s="1">
         <v>207</v>
       </c>
-      <c r="B208" s="2">
+      <c r="B208" s="1">
         <v>4000</v>
       </c>
       <c r="C208" s="1">
@@ -3384,7 +3373,7 @@
       <c r="A209" s="1">
         <v>208</v>
       </c>
-      <c r="B209" s="2">
+      <c r="B209" s="1">
         <v>4000</v>
       </c>
       <c r="C209" s="1">
@@ -3396,7 +3385,7 @@
       <c r="A210" s="1">
         <v>209</v>
       </c>
-      <c r="B210" s="2">
+      <c r="B210" s="1">
         <v>4000</v>
       </c>
       <c r="C210" s="1">
@@ -3408,7 +3397,7 @@
       <c r="A211" s="1">
         <v>210</v>
       </c>
-      <c r="B211" s="2">
+      <c r="B211" s="1">
         <v>4000</v>
       </c>
       <c r="C211" s="1">
@@ -3420,7 +3409,7 @@
       <c r="A212" s="1">
         <v>211</v>
       </c>
-      <c r="B212" s="2">
+      <c r="B212" s="1">
         <v>4000</v>
       </c>
       <c r="C212" s="1">
@@ -3432,7 +3421,7 @@
       <c r="A213" s="1">
         <v>212</v>
       </c>
-      <c r="B213" s="2">
+      <c r="B213" s="1">
         <v>4400</v>
       </c>
       <c r="C213" s="1">
@@ -3444,7 +3433,7 @@
       <c r="A214" s="1">
         <v>213</v>
       </c>
-      <c r="B214" s="2">
+      <c r="B214" s="1">
         <v>4400</v>
       </c>
       <c r="C214" s="1">
@@ -3456,7 +3445,7 @@
       <c r="A215" s="1">
         <v>214</v>
       </c>
-      <c r="B215" s="2">
+      <c r="B215" s="1">
         <v>4400</v>
       </c>
       <c r="C215" s="1">
@@ -3468,7 +3457,7 @@
       <c r="A216" s="1">
         <v>215</v>
       </c>
-      <c r="B216" s="2">
+      <c r="B216" s="1">
         <v>4400</v>
       </c>
       <c r="C216" s="1">
@@ -3480,7 +3469,7 @@
       <c r="A217" s="1">
         <v>216</v>
       </c>
-      <c r="B217" s="2">
+      <c r="B217" s="1">
         <v>4400</v>
       </c>
       <c r="C217" s="1">
@@ -3492,7 +3481,7 @@
       <c r="A218" s="1">
         <v>217</v>
       </c>
-      <c r="B218" s="2">
+      <c r="B218" s="1">
         <v>4400</v>
       </c>
       <c r="C218" s="1">
@@ -3504,7 +3493,7 @@
       <c r="A219" s="1">
         <v>218</v>
       </c>
-      <c r="B219" s="2">
+      <c r="B219" s="1">
         <v>4400</v>
       </c>
       <c r="C219" s="1">
@@ -3516,7 +3505,7 @@
       <c r="A220" s="1">
         <v>219</v>
       </c>
-      <c r="B220" s="2">
+      <c r="B220" s="1">
         <v>4400</v>
       </c>
       <c r="C220" s="1">
@@ -3528,7 +3517,7 @@
       <c r="A221" s="1">
         <v>220</v>
       </c>
-      <c r="B221" s="2">
+      <c r="B221" s="1">
         <v>4400</v>
       </c>
       <c r="C221" s="1">
@@ -3540,7 +3529,7 @@
       <c r="A222" s="1">
         <v>221</v>
       </c>
-      <c r="B222" s="2">
+      <c r="B222" s="1">
         <v>4400</v>
       </c>
       <c r="C222" s="1">
@@ -3552,7 +3541,7 @@
       <c r="A223" s="1">
         <v>222</v>
       </c>
-      <c r="B223" s="2">
+      <c r="B223" s="1">
         <v>4800</v>
       </c>
       <c r="C223" s="1">
@@ -3564,7 +3553,7 @@
       <c r="A224" s="1">
         <v>223</v>
       </c>
-      <c r="B224" s="2">
+      <c r="B224" s="1">
         <v>4800</v>
       </c>
       <c r="C224" s="1">
@@ -3576,7 +3565,7 @@
       <c r="A225" s="1">
         <v>224</v>
       </c>
-      <c r="B225" s="2">
+      <c r="B225" s="1">
         <v>4800</v>
       </c>
       <c r="C225" s="1">
@@ -3588,7 +3577,7 @@
       <c r="A226" s="1">
         <v>225</v>
       </c>
-      <c r="B226" s="2">
+      <c r="B226" s="1">
         <v>4800</v>
       </c>
       <c r="C226" s="1">
@@ -3600,7 +3589,7 @@
       <c r="A227" s="1">
         <v>226</v>
       </c>
-      <c r="B227" s="2">
+      <c r="B227" s="1">
         <v>4800</v>
       </c>
       <c r="C227" s="1">
@@ -3612,7 +3601,7 @@
       <c r="A228" s="1">
         <v>227</v>
       </c>
-      <c r="B228" s="2">
+      <c r="B228" s="1">
         <v>4800</v>
       </c>
       <c r="C228" s="1">
@@ -3624,7 +3613,7 @@
       <c r="A229" s="1">
         <v>228</v>
       </c>
-      <c r="B229" s="2">
+      <c r="B229" s="1">
         <v>4800</v>
       </c>
       <c r="C229" s="1">
@@ -3636,7 +3625,7 @@
       <c r="A230" s="1">
         <v>229</v>
       </c>
-      <c r="B230" s="2">
+      <c r="B230" s="1">
         <v>4800</v>
       </c>
       <c r="C230" s="1">
@@ -3648,7 +3637,7 @@
       <c r="A231" s="1">
         <v>230</v>
       </c>
-      <c r="B231" s="2">
+      <c r="B231" s="1">
         <v>4800</v>
       </c>
       <c r="C231" s="1">
@@ -3660,7 +3649,7 @@
       <c r="A232" s="1">
         <v>231</v>
       </c>
-      <c r="B232" s="2">
+      <c r="B232" s="1">
         <v>4800</v>
       </c>
       <c r="C232" s="1">
@@ -3672,7 +3661,7 @@
       <c r="A233" s="1">
         <v>232</v>
       </c>
-      <c r="B233" s="2">
+      <c r="B233" s="1">
         <v>5200</v>
       </c>
       <c r="C233" s="1">
@@ -3684,7 +3673,7 @@
       <c r="A234" s="1">
         <v>233</v>
       </c>
-      <c r="B234" s="2">
+      <c r="B234" s="1">
         <v>5200</v>
       </c>
       <c r="C234" s="1">
@@ -3696,7 +3685,7 @@
       <c r="A235" s="1">
         <v>234</v>
       </c>
-      <c r="B235" s="2">
+      <c r="B235" s="1">
         <v>5200</v>
       </c>
       <c r="C235" s="1">
@@ -3708,7 +3697,7 @@
       <c r="A236" s="1">
         <v>235</v>
       </c>
-      <c r="B236" s="2">
+      <c r="B236" s="1">
         <v>5200</v>
       </c>
       <c r="C236" s="1">
@@ -3720,7 +3709,7 @@
       <c r="A237" s="1">
         <v>236</v>
       </c>
-      <c r="B237" s="2">
+      <c r="B237" s="1">
         <v>5200</v>
       </c>
       <c r="C237" s="1">
@@ -3732,7 +3721,7 @@
       <c r="A238" s="1">
         <v>237</v>
       </c>
-      <c r="B238" s="2">
+      <c r="B238" s="1">
         <v>5200</v>
       </c>
       <c r="C238" s="1">
@@ -3744,7 +3733,7 @@
       <c r="A239" s="1">
         <v>238</v>
       </c>
-      <c r="B239" s="2">
+      <c r="B239" s="1">
         <v>5200</v>
       </c>
       <c r="C239" s="1">
@@ -3756,7 +3745,7 @@
       <c r="A240" s="1">
         <v>239</v>
       </c>
-      <c r="B240" s="2">
+      <c r="B240" s="1">
         <v>5200</v>
       </c>
       <c r="C240" s="1">
@@ -3768,7 +3757,7 @@
       <c r="A241" s="1">
         <v>240</v>
       </c>
-      <c r="B241" s="2">
+      <c r="B241" s="1">
         <v>5200</v>
       </c>
       <c r="C241" s="1">
@@ -3780,7 +3769,7 @@
       <c r="A242" s="1">
         <v>241</v>
       </c>
-      <c r="B242" s="2">
+      <c r="B242" s="1">
         <v>5200</v>
       </c>
       <c r="C242" s="1">
@@ -3792,7 +3781,7 @@
       <c r="A243" s="1">
         <v>242</v>
       </c>
-      <c r="B243" s="2">
+      <c r="B243" s="1">
         <v>5600</v>
       </c>
       <c r="C243" s="1">
@@ -3804,7 +3793,7 @@
       <c r="A244" s="1">
         <v>243</v>
       </c>
-      <c r="B244" s="2">
+      <c r="B244" s="1">
         <v>5600</v>
       </c>
       <c r="C244" s="1">
@@ -3816,7 +3805,7 @@
       <c r="A245" s="1">
         <v>244</v>
       </c>
-      <c r="B245" s="2">
+      <c r="B245" s="1">
         <v>5600</v>
       </c>
       <c r="C245" s="1">
@@ -3828,7 +3817,7 @@
       <c r="A246" s="1">
         <v>245</v>
       </c>
-      <c r="B246" s="2">
+      <c r="B246" s="1">
         <v>5600</v>
       </c>
       <c r="C246" s="1">
@@ -3840,7 +3829,7 @@
       <c r="A247" s="1">
         <v>246</v>
       </c>
-      <c r="B247" s="2">
+      <c r="B247" s="1">
         <v>5600</v>
       </c>
       <c r="C247" s="1">
@@ -3852,7 +3841,7 @@
       <c r="A248" s="1">
         <v>247</v>
       </c>
-      <c r="B248" s="2">
+      <c r="B248" s="1">
         <v>5600</v>
       </c>
       <c r="C248" s="1">
@@ -3864,7 +3853,7 @@
       <c r="A249" s="1">
         <v>248</v>
       </c>
-      <c r="B249" s="2">
+      <c r="B249" s="1">
         <v>5600</v>
       </c>
       <c r="C249" s="1">
@@ -3876,7 +3865,7 @@
       <c r="A250" s="1">
         <v>249</v>
       </c>
-      <c r="B250" s="2">
+      <c r="B250" s="1">
         <v>5600</v>
       </c>
       <c r="C250" s="1">
@@ -3888,7 +3877,7 @@
       <c r="A251" s="1">
         <v>250</v>
       </c>
-      <c r="B251" s="2">
+      <c r="B251" s="1">
         <v>5600</v>
       </c>
       <c r="C251" s="1">
@@ -3900,7 +3889,7 @@
       <c r="A252" s="1">
         <v>251</v>
       </c>
-      <c r="B252" s="2">
+      <c r="B252" s="1">
         <v>5600</v>
       </c>
       <c r="C252" s="1">
@@ -3912,7 +3901,7 @@
       <c r="A253" s="1">
         <v>252</v>
       </c>
-      <c r="B253" s="2">
+      <c r="B253" s="1">
         <v>6000</v>
       </c>
       <c r="C253" s="1">
@@ -3924,7 +3913,7 @@
       <c r="A254" s="1">
         <v>253</v>
       </c>
-      <c r="B254" s="2">
+      <c r="B254" s="1">
         <v>6000</v>
       </c>
       <c r="C254" s="1">
@@ -3936,7 +3925,7 @@
       <c r="A255" s="1">
         <v>254</v>
       </c>
-      <c r="B255" s="2">
+      <c r="B255" s="1">
         <v>6000</v>
       </c>
       <c r="C255" s="1">
@@ -3948,7 +3937,7 @@
       <c r="A256" s="1">
         <v>255</v>
       </c>
-      <c r="B256" s="2">
+      <c r="B256" s="1">
         <v>6000</v>
       </c>
       <c r="C256" s="1">
@@ -3960,7 +3949,7 @@
       <c r="A257" s="1">
         <v>256</v>
       </c>
-      <c r="B257" s="2">
+      <c r="B257" s="1">
         <v>6000</v>
       </c>
       <c r="C257" s="1">
@@ -3972,7 +3961,7 @@
       <c r="A258" s="1">
         <v>257</v>
       </c>
-      <c r="B258" s="2">
+      <c r="B258" s="1">
         <v>6000</v>
       </c>
       <c r="C258" s="1">
@@ -3984,7 +3973,7 @@
       <c r="A259" s="1">
         <v>258</v>
       </c>
-      <c r="B259" s="2">
+      <c r="B259" s="1">
         <v>6000</v>
       </c>
       <c r="C259" s="1">
@@ -3996,7 +3985,7 @@
       <c r="A260" s="1">
         <v>259</v>
       </c>
-      <c r="B260" s="2">
+      <c r="B260" s="1">
         <v>6000</v>
       </c>
       <c r="C260" s="1">
@@ -4008,7 +3997,7 @@
       <c r="A261" s="1">
         <v>260</v>
       </c>
-      <c r="B261" s="2">
+      <c r="B261" s="1">
         <v>6000</v>
       </c>
       <c r="C261" s="1">
@@ -4020,7 +4009,7 @@
       <c r="A262" s="1">
         <v>261</v>
       </c>
-      <c r="B262" s="2">
+      <c r="B262" s="1">
         <v>6000</v>
       </c>
       <c r="C262" s="1">
@@ -4032,7 +4021,7 @@
       <c r="A263" s="1">
         <v>262</v>
       </c>
-      <c r="B263" s="2">
+      <c r="B263" s="1">
         <v>6500</v>
       </c>
       <c r="C263" s="1">
@@ -4044,7 +4033,7 @@
       <c r="A264" s="1">
         <v>263</v>
       </c>
-      <c r="B264" s="2">
+      <c r="B264" s="1">
         <v>6500</v>
       </c>
       <c r="C264" s="1">
@@ -4056,7 +4045,7 @@
       <c r="A265" s="1">
         <v>264</v>
       </c>
-      <c r="B265" s="2">
+      <c r="B265" s="1">
         <v>6500</v>
       </c>
       <c r="C265" s="1">
@@ -4068,7 +4057,7 @@
       <c r="A266" s="1">
         <v>265</v>
       </c>
-      <c r="B266" s="2">
+      <c r="B266" s="1">
         <v>6500</v>
       </c>
       <c r="C266" s="1">
@@ -4080,7 +4069,7 @@
       <c r="A267" s="1">
         <v>266</v>
       </c>
-      <c r="B267" s="2">
+      <c r="B267" s="1">
         <v>6500</v>
       </c>
       <c r="C267" s="1">
@@ -4092,7 +4081,7 @@
       <c r="A268" s="1">
         <v>267</v>
       </c>
-      <c r="B268" s="2">
+      <c r="B268" s="1">
         <v>6500</v>
       </c>
       <c r="C268" s="1">
@@ -4104,7 +4093,7 @@
       <c r="A269" s="1">
         <v>268</v>
       </c>
-      <c r="B269" s="2">
+      <c r="B269" s="1">
         <v>6500</v>
       </c>
       <c r="C269" s="1">
@@ -4116,7 +4105,7 @@
       <c r="A270" s="1">
         <v>269</v>
       </c>
-      <c r="B270" s="2">
+      <c r="B270" s="1">
         <v>6500</v>
       </c>
       <c r="C270" s="1">
@@ -4128,7 +4117,7 @@
       <c r="A271" s="1">
         <v>270</v>
       </c>
-      <c r="B271" s="2">
+      <c r="B271" s="1">
         <v>6500</v>
       </c>
       <c r="C271" s="1">
@@ -4140,7 +4129,7 @@
       <c r="A272" s="1">
         <v>271</v>
       </c>
-      <c r="B272" s="2">
+      <c r="B272" s="1">
         <v>6500</v>
       </c>
       <c r="C272" s="1">
@@ -4152,7 +4141,7 @@
       <c r="A273" s="1">
         <v>272</v>
       </c>
-      <c r="B273" s="2">
+      <c r="B273" s="1">
         <v>7000</v>
       </c>
       <c r="C273" s="1">
@@ -4164,7 +4153,7 @@
       <c r="A274" s="1">
         <v>273</v>
       </c>
-      <c r="B274" s="2">
+      <c r="B274" s="1">
         <v>7000</v>
       </c>
       <c r="C274" s="1">
@@ -4176,7 +4165,7 @@
       <c r="A275" s="1">
         <v>274</v>
       </c>
-      <c r="B275" s="2">
+      <c r="B275" s="1">
         <v>7000</v>
       </c>
       <c r="C275" s="1">
@@ -4188,7 +4177,7 @@
       <c r="A276" s="1">
         <v>275</v>
       </c>
-      <c r="B276" s="2">
+      <c r="B276" s="1">
         <v>7000</v>
       </c>
       <c r="C276" s="1">
@@ -4200,7 +4189,7 @@
       <c r="A277" s="1">
         <v>276</v>
       </c>
-      <c r="B277" s="2">
+      <c r="B277" s="1">
         <v>7000</v>
       </c>
       <c r="C277" s="1">
@@ -4212,7 +4201,7 @@
       <c r="A278" s="1">
         <v>277</v>
       </c>
-      <c r="B278" s="2">
+      <c r="B278" s="1">
         <v>7000</v>
       </c>
       <c r="C278" s="1">
@@ -4224,7 +4213,7 @@
       <c r="A279" s="1">
         <v>278</v>
       </c>
-      <c r="B279" s="2">
+      <c r="B279" s="1">
         <v>7000</v>
       </c>
       <c r="C279" s="1">
@@ -4236,7 +4225,7 @@
       <c r="A280" s="1">
         <v>279</v>
       </c>
-      <c r="B280" s="2">
+      <c r="B280" s="1">
         <v>7000</v>
       </c>
       <c r="C280" s="1">
@@ -4248,7 +4237,7 @@
       <c r="A281" s="1">
         <v>280</v>
       </c>
-      <c r="B281" s="2">
+      <c r="B281" s="1">
         <v>7000</v>
       </c>
       <c r="C281" s="1">
@@ -4260,7 +4249,7 @@
       <c r="A282" s="1">
         <v>281</v>
       </c>
-      <c r="B282" s="2">
+      <c r="B282" s="1">
         <v>7000</v>
       </c>
       <c r="C282" s="1">
@@ -4272,7 +4261,7 @@
       <c r="A283" s="1">
         <v>282</v>
       </c>
-      <c r="B283" s="2">
+      <c r="B283" s="1">
         <v>7500</v>
       </c>
       <c r="C283" s="1">
@@ -4284,7 +4273,7 @@
       <c r="A284" s="1">
         <v>283</v>
       </c>
-      <c r="B284" s="2">
+      <c r="B284" s="1">
         <v>7500</v>
       </c>
       <c r="C284" s="1">
@@ -4296,7 +4285,7 @@
       <c r="A285" s="1">
         <v>284</v>
       </c>
-      <c r="B285" s="2">
+      <c r="B285" s="1">
         <v>7500</v>
       </c>
       <c r="C285" s="1">
@@ -4308,7 +4297,7 @@
       <c r="A286" s="1">
         <v>285</v>
       </c>
-      <c r="B286" s="2">
+      <c r="B286" s="1">
         <v>7500</v>
       </c>
       <c r="C286" s="1">
@@ -4320,7 +4309,7 @@
       <c r="A287" s="1">
         <v>286</v>
       </c>
-      <c r="B287" s="2">
+      <c r="B287" s="1">
         <v>7500</v>
       </c>
       <c r="C287" s="1">
@@ -4332,7 +4321,7 @@
       <c r="A288" s="1">
         <v>287</v>
       </c>
-      <c r="B288" s="2">
+      <c r="B288" s="1">
         <v>7500</v>
       </c>
       <c r="C288" s="1">
@@ -4344,7 +4333,7 @@
       <c r="A289" s="1">
         <v>288</v>
       </c>
-      <c r="B289" s="2">
+      <c r="B289" s="1">
         <v>7500</v>
       </c>
       <c r="C289" s="1">
@@ -4356,7 +4345,7 @@
       <c r="A290" s="1">
         <v>289</v>
       </c>
-      <c r="B290" s="2">
+      <c r="B290" s="1">
         <v>7500</v>
       </c>
       <c r="C290" s="1">
@@ -4368,7 +4357,7 @@
       <c r="A291" s="1">
         <v>290</v>
       </c>
-      <c r="B291" s="2">
+      <c r="B291" s="1">
         <v>7500</v>
       </c>
       <c r="C291" s="1">
@@ -4380,7 +4369,7 @@
       <c r="A292" s="1">
         <v>291</v>
       </c>
-      <c r="B292" s="2">
+      <c r="B292" s="1">
         <v>7500</v>
       </c>
       <c r="C292" s="1">
@@ -4392,7 +4381,7 @@
       <c r="A293" s="1">
         <v>292</v>
       </c>
-      <c r="B293" s="2">
+      <c r="B293" s="1">
         <v>8000</v>
       </c>
       <c r="C293" s="1">
@@ -4404,7 +4393,7 @@
       <c r="A294" s="1">
         <v>293</v>
       </c>
-      <c r="B294" s="2">
+      <c r="B294" s="1">
         <v>8000</v>
       </c>
       <c r="C294" s="1">
@@ -4416,7 +4405,7 @@
       <c r="A295" s="1">
         <v>294</v>
       </c>
-      <c r="B295" s="2">
+      <c r="B295" s="1">
         <v>8000</v>
       </c>
       <c r="C295" s="1">
@@ -4428,7 +4417,7 @@
       <c r="A296" s="1">
         <v>295</v>
       </c>
-      <c r="B296" s="2">
+      <c r="B296" s="1">
         <v>8000</v>
       </c>
       <c r="C296" s="1">
@@ -4440,7 +4429,7 @@
       <c r="A297" s="1">
         <v>296</v>
       </c>
-      <c r="B297" s="2">
+      <c r="B297" s="1">
         <v>8000</v>
       </c>
       <c r="C297" s="1">
@@ -4452,7 +4441,7 @@
       <c r="A298" s="1">
         <v>297</v>
       </c>
-      <c r="B298" s="2">
+      <c r="B298" s="1">
         <v>8000</v>
       </c>
       <c r="C298" s="1">
@@ -4464,7 +4453,7 @@
       <c r="A299" s="1">
         <v>298</v>
       </c>
-      <c r="B299" s="2">
+      <c r="B299" s="1">
         <v>8000</v>
       </c>
       <c r="C299" s="1">
@@ -4476,7 +4465,7 @@
       <c r="A300" s="1">
         <v>299</v>
       </c>
-      <c r="B300" s="2">
+      <c r="B300" s="1">
         <v>8000</v>
       </c>
       <c r="C300" s="1">
@@ -4488,7 +4477,7 @@
       <c r="A301" s="1">
         <v>300</v>
       </c>
-      <c r="B301" s="2">
+      <c r="B301" s="1">
         <v>8000</v>
       </c>
       <c r="C301" s="1">
@@ -4500,7 +4489,7 @@
       <c r="A302" s="1">
         <v>301</v>
       </c>
-      <c r="B302" s="2">
+      <c r="B302" s="1">
         <v>8000</v>
       </c>
       <c r="C302" s="1">

</xml_diff>